<commit_message>
v9 - extra participants
</commit_message>
<xml_diff>
--- a/occupations.xlsx
+++ b/occupations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parti\Projects\occupational-gender-bias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14DB2F71-B6D7-4419-B7E5-54024B8C630C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6216A19F-FA08-449F-B664-68068AE79280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="825" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="825" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="occupations" sheetId="1" r:id="rId1"/>
@@ -752,9 +752,6 @@
   </cellStyles>
   <dxfs count="32">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -894,6 +891,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -934,32 +934,32 @@
     <tableColumn id="17" xr3:uid="{A874A889-7532-45D4-B042-5A57A6832C05}" name="r" dataDxfId="27">
       <calculatedColumnFormula>RAND()</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{97EE8D88-168B-4084-A4F7-3D90DC6E0437}" name="service" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{A494C8E6-F914-428C-8272-43E167056E6E}" name="en" dataDxfId="26"/>
-    <tableColumn id="29" xr3:uid="{919903A9-489F-4E4F-ADD1-D9FE34CBD814}" name="hu" dataDxfId="25"/>
-    <tableColumn id="30" xr3:uid="{A7971DCE-3EEE-4AC4-B952-2B4AC52EB4E5}" name="item_hu" dataDxfId="24"/>
-    <tableColumn id="31" xr3:uid="{9ED8DFFE-0B05-4EB4-8905-544B1AEC595A}" name="zh" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{1B4C41A2-3CB1-4152-B81F-485D7760D63F}" name="item_zh" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{D5BAA5F6-6A6C-4A62-87E9-103082EBCD62}" name="lechat_hu" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{759290F1-F27B-4ACB-8412-511B2D39315D}" name="lechat_hu_std" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{4A32F8C1-359D-4C9E-8195-02A92870A71F}" name="copilot_hu" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{FAED1BDE-D712-4736-B7E1-9432AA7B56C5}" name="copilot_hu_std" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{5D26EFD2-BF07-4806-8FBB-9F219CC0741B}" name="chatgpt_hu" dataDxfId="17"/>
-    <tableColumn id="16" xr3:uid="{A5A18E72-2DF3-4103-ABBE-8E8734EA738F}" name="chatgpt_hu_std" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{F1FF7BC1-AC09-41A0-800C-522EDB48326B}" name="deepseek_hu" dataDxfId="15"/>
-    <tableColumn id="19" xr3:uid="{793655E4-E741-4893-982C-6F8D70FC4888}" name="deepseek_hu_std" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{F30252C1-B7F3-463E-8FA4-511299C5F348}" name="gemini_hu" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{E88D4172-7B47-4387-A704-62B6A3AF195F}" name="gemini_hu_std" dataDxfId="12"/>
-    <tableColumn id="24" xr3:uid="{13C47BE2-8249-4469-A639-66EC0E40FD3E}" name="lechat_zh" dataDxfId="11"/>
-    <tableColumn id="23" xr3:uid="{0AA50B4C-75C2-49C4-B969-6A8E636B807E}" name="lechat_zh_std" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{18983B9A-B075-414F-8D87-3F5A25C293D4}" name="copilot_zh" dataDxfId="9"/>
-    <tableColumn id="25" xr3:uid="{123F14B8-5B61-4C77-88B9-777EBB7C5B66}" name="copilot_zh_std" dataDxfId="8"/>
-    <tableColumn id="18" xr3:uid="{9ABFFE5E-A61F-4A56-9BD3-5CB3EAEDAC22}" name="chatgpt_zh" dataDxfId="7"/>
-    <tableColumn id="26" xr3:uid="{BCA942D6-2851-4C1D-A977-396C0CAD2878}" name="chatgpt_zh_std" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{A39B0E6C-C60A-405D-9049-F1F4B921C73F}" name="deepseek_zh" dataDxfId="5"/>
-    <tableColumn id="27" xr3:uid="{01166CB3-78C0-4F10-83EF-CE4646B82547}" name="deepseek_zh_std" dataDxfId="4"/>
-    <tableColumn id="21" xr3:uid="{09D3EAFF-C9B4-4CCD-803F-7FC1828A805E}" name="gemini_zh" dataDxfId="3"/>
-    <tableColumn id="28" xr3:uid="{540117C0-7A45-4A5D-8D55-14A76C85A71A}" name="gemini_zh_std" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{97EE8D88-168B-4084-A4F7-3D90DC6E0437}" name="service" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{A494C8E6-F914-428C-8272-43E167056E6E}" name="en" dataDxfId="25"/>
+    <tableColumn id="29" xr3:uid="{919903A9-489F-4E4F-ADD1-D9FE34CBD814}" name="hu" dataDxfId="24"/>
+    <tableColumn id="30" xr3:uid="{A7971DCE-3EEE-4AC4-B952-2B4AC52EB4E5}" name="item_hu" dataDxfId="23"/>
+    <tableColumn id="31" xr3:uid="{9ED8DFFE-0B05-4EB4-8905-544B1AEC595A}" name="zh" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{1B4C41A2-3CB1-4152-B81F-485D7760D63F}" name="item_zh" dataDxfId="21"/>
+    <tableColumn id="14" xr3:uid="{D5BAA5F6-6A6C-4A62-87E9-103082EBCD62}" name="lechat_hu" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{759290F1-F27B-4ACB-8412-511B2D39315D}" name="lechat_hu_std" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{4A32F8C1-359D-4C9E-8195-02A92870A71F}" name="copilot_hu" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{FAED1BDE-D712-4736-B7E1-9432AA7B56C5}" name="copilot_hu_std" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{5D26EFD2-BF07-4806-8FBB-9F219CC0741B}" name="chatgpt_hu" dataDxfId="16"/>
+    <tableColumn id="16" xr3:uid="{A5A18E72-2DF3-4103-ABBE-8E8734EA738F}" name="chatgpt_hu_std" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{F1FF7BC1-AC09-41A0-800C-522EDB48326B}" name="deepseek_hu" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{793655E4-E741-4893-982C-6F8D70FC4888}" name="deepseek_hu_std" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{F30252C1-B7F3-463E-8FA4-511299C5F348}" name="gemini_hu" dataDxfId="12"/>
+    <tableColumn id="22" xr3:uid="{E88D4172-7B47-4387-A704-62B6A3AF195F}" name="gemini_hu_std" dataDxfId="11"/>
+    <tableColumn id="24" xr3:uid="{13C47BE2-8249-4469-A639-66EC0E40FD3E}" name="lechat_zh" dataDxfId="10"/>
+    <tableColumn id="23" xr3:uid="{0AA50B4C-75C2-49C4-B969-6A8E636B807E}" name="lechat_zh_std" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{18983B9A-B075-414F-8D87-3F5A25C293D4}" name="copilot_zh" dataDxfId="8"/>
+    <tableColumn id="25" xr3:uid="{123F14B8-5B61-4C77-88B9-777EBB7C5B66}" name="copilot_zh_std" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{9ABFFE5E-A61F-4A56-9BD3-5CB3EAEDAC22}" name="chatgpt_zh" dataDxfId="6"/>
+    <tableColumn id="26" xr3:uid="{BCA942D6-2851-4C1D-A977-396C0CAD2878}" name="chatgpt_zh_std" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{A39B0E6C-C60A-405D-9049-F1F4B921C73F}" name="deepseek_zh" dataDxfId="4"/>
+    <tableColumn id="27" xr3:uid="{01166CB3-78C0-4F10-83EF-CE4646B82547}" name="deepseek_zh_std" dataDxfId="3"/>
+    <tableColumn id="21" xr3:uid="{09D3EAFF-C9B4-4CCD-803F-7FC1828A805E}" name="gemini_zh" dataDxfId="2"/>
+    <tableColumn id="28" xr3:uid="{540117C0-7A45-4A5D-8D55-14A76C85A71A}" name="gemini_zh_std" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C2" s="4">
         <f t="shared" ref="C2:C33" ca="1" si="0">RAND()</f>
-        <v>0.38222186627203114</v>
+        <v>0.85943030657802322</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" t="s">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.49833329861652165</v>
+        <v>0.38708481545833839</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" t="s">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="C4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.54258934921252888</v>
+        <v>3.1755750817918926E-2</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" t="s">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="C5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>5.3284754081942332E-2</v>
+        <v>0.96082274315782246</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" t="s">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="C6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.1884759825897776</v>
+        <v>0.87000640023742692</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" t="s">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="C7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73159141848714782</v>
+        <v>1.5698810745665148E-2</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" t="s">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="C8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.7190640120054651</v>
+        <v>0.21252852963534719</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" t="s">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="C9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.98127753013503038</v>
+        <v>0.6508542517810284</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" t="s">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.29453137215569669</v>
+        <v>0.18791451621465083</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" t="s">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="C11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44872009265870982</v>
+        <v>0.43766241365658154</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" t="s">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="C12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.2899758953061865</v>
+        <v>0.69847058357960534</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" t="s">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="C13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>9.0892628959652555E-2</v>
+        <v>0.3707557703316493</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" t="s">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="C14" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.80978269760174149</v>
+        <v>0.95360805385962244</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" t="s">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="C15" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.36049955427220459</v>
+        <v>2.8936632638175808E-2</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" t="s">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C16" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.11422688931518377</v>
+        <v>0.77014582128354347</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" t="s">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="C17" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>8.9728609495878686E-2</v>
+        <v>0.66681205980303515</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" t="s">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="C18" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.42540443951753149</v>
+        <v>3.0419163870829324E-2</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" t="s">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="C19" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.12254010815310823</v>
+        <v>0.14800263379243472</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" t="s">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="C20" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.61124010027983033</v>
+        <v>0.51717150701019665</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" t="s">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="C21" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.63862603306140509</v>
+        <v>0.28990262460281391</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" t="s">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="C22" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.18225626008841567</v>
+        <v>0.59363802635255347</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" t="s">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="C23" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3.8923318392179551E-2</v>
+        <v>0.2596608849512464</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" t="s">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="C24" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.50786871101767328</v>
+        <v>0.64349530181527714</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" t="s">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="C25" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.64992419004321789</v>
+        <v>0.40179288809041414</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" t="s">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="C26" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.93263958888478293</v>
+        <v>0.72076276132646888</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" t="s">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="C27" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.84159449305786616</v>
+        <v>0.75940368088687804</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" t="s">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="C28" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.6605383144470629</v>
+        <v>0.2381729165628369</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" t="s">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="C29" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.94859686314379243</v>
+        <v>0.99698942055445805</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" t="s">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="C30" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.61119908724147309</v>
+        <v>0.10286211975493942</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" t="s">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="C31" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73340681953930364</v>
+        <v>2.7530396681456848E-2</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" t="s">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="C32" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.61650289543394754</v>
+        <v>0.97063418565785908</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" t="s">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="C33" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0.4224407237224761</v>
+        <v>0.41751094636683239</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" t="s">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="C34" s="4">
         <f t="shared" ref="C34:C60" ca="1" si="1">RAND()</f>
-        <v>9.6590244446947193E-2</v>
+        <v>0.9722584954722111</v>
       </c>
       <c r="D34" s="4"/>
       <c r="E34" t="s">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="C35" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75233790229423336</v>
+        <v>0.43465131183043704</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" t="s">
@@ -4480,7 +4480,7 @@
       </c>
       <c r="C36" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.37905939422339685</v>
+        <v>0.94232040157541774</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" t="s">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C37" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.57914476532020154</v>
+        <v>0.78319325383963234</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" t="s">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="C38" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.61384000463604271</v>
+        <v>0.74488697706124241</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" t="s">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="C39" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.92913636099936336</v>
+        <v>0.41087101982929697</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" t="s">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="C40" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.83873297982506823</v>
+        <v>0.76757562859755868</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" t="s">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="C41" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>9.9628881726652518E-2</v>
+        <v>0.34332065682880841</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" t="s">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="C42" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.13943755357800791</v>
+        <v>0.46860911881006573</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" t="s">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="C43" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.79580316116749994</v>
+        <v>0.51889141623674373</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" t="s">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="C44" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.37498084365287798</v>
+        <v>0.82266140760107243</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" t="s">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="C45" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.41392932711097674</v>
+        <v>7.7573753190827932E-2</v>
       </c>
       <c r="D45" s="4"/>
       <c r="E45" t="s">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="C46" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.30504986941276346</v>
+        <v>0.39046552007320745</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" t="s">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="C47" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>1.4306998694183837E-2</v>
+        <v>0.76254053706386393</v>
       </c>
       <c r="D47" s="4"/>
       <c r="E47" t="s">
@@ -5560,7 +5560,7 @@
       </c>
       <c r="C48" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>5.0158770822335219E-2</v>
+        <v>0.11050351468306296</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" t="s">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="C49" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>8.9311632578731093E-2</v>
+        <v>0.1764464893881923</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" t="s">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="C50" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>3.9449733166332601E-2</v>
+        <v>0.89472555143530252</v>
       </c>
       <c r="D50" s="4"/>
       <c r="E50" t="s">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="C51" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.3973026969418928</v>
+        <v>0.48349499706344679</v>
       </c>
       <c r="D51" s="4"/>
       <c r="E51" t="s">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="C52" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74153759772342653</v>
+        <v>0.20627698363672853</v>
       </c>
       <c r="D52" s="4"/>
       <c r="E52" t="s">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="C53" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.61723873194395729</v>
+        <v>0.90305759576454558</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" t="s">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="C54" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86846159516572019</v>
+        <v>0.68490146055378298</v>
       </c>
       <c r="D54" s="4"/>
       <c r="E54" t="s">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="C55" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.45657654781532142</v>
+        <v>0.8911694182129104</v>
       </c>
       <c r="D55" s="4"/>
       <c r="E55" t="s">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="C56" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72056651478880718</v>
+        <v>0.90540546578100722</v>
       </c>
       <c r="D56" s="4"/>
       <c r="E56" t="s">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="C57" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>2.9015323888088029E-2</v>
+        <v>0.57707139566393517</v>
       </c>
       <c r="D57" s="4"/>
       <c r="E57" t="s">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="C58" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.87952636490060487</v>
+        <v>0.32594252227319997</v>
       </c>
       <c r="D58" s="4"/>
       <c r="E58" t="s">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="C59" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>9.6282375395473463E-2</v>
+        <v>0.7323562386559529</v>
       </c>
       <c r="D59" s="4"/>
       <c r="E59" t="s">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C60" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.79281912998821835</v>
+        <v>0.31164621853682128</v>
       </c>
       <c r="D60" s="4"/>
       <c r="E60" t="s">
@@ -6724,7 +6724,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="E1:F1048576 H1:H1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>